<commit_message>
Adopt matrix v8: AGG Reflation cell re-places leverage (QQQ 1x + ERX 2x tilt)
- matrix.py: MATRIX_VERSION v8; AGG R = QQQ .30 + ERX/GDX/DBC momentum trio; VAGG/MOD/CONS unchanged
- paper_logger.current_allocations(): re-resolves older-version ledger rows from stored signals
  under the current matrix (append-only ledger untouched); manual order tools use it,
  the automated executor reads ledger rows as-is
- orders_workbook --tier; RotationOrders.xlsx regenerated (AGG, v8 restated from Sept signals)
- evidence.json / projection_stats.json / GrowthProjection.xlsx regenerated under v8
  (AGG +24.6% / 1.26 / -34.2%)
- InvestmentSystemOverview.docx AGG row updated; TESTS.md adopted #14; PORTFOLIOS/DEPLOYMENT notes
- 94 tests passing

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1223,7 +1223,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Age-based risk glide with regime-conditional return engine  |  Backtest Jun 2007–Aug 2026  |  Prepared August 26, 2026  |  Forward ledger live</t>
+          <t>Age-based risk glide with regime-conditional return engine  |  Backtest Jun 2007–Aug 2026  |  Prepared September 09, 2026  |  Forward ledger live</t>
         </is>
       </c>
     </row>
@@ -1836,34 +1836,34 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>0.242</v>
+        <v>0.2464</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>1.2306</v>
+        <v>1.2614</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>0.9532</v>
+        <v>0.9626</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>-0.3342</v>
+        <v>-0.3422</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>0.6317</v>
+        <v>0.6035</v>
       </c>
       <c r="G8" s="18" t="n">
         <v>0.3038</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>0.8095</v>
+        <v>0.6695</v>
       </c>
       <c r="I8" s="18" t="n">
-        <v>-0.2478</v>
+        <v>-0.1363</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.5212</v>
+        <v>0.5427</v>
       </c>
       <c r="K8" s="18" t="n">
-        <v>0.217</v>
+        <v>0.3711</v>
       </c>
     </row>
     <row r="9">
@@ -18394,7 +18394,7 @@
         <v>0.03406</v>
       </c>
       <c r="C8" s="55" t="n">
-        <v>0.01229</v>
+        <v>0.01308</v>
       </c>
       <c r="D8" s="55" t="n">
         <v>0.00804</v>
@@ -18503,7 +18503,7 @@
         <v>0.09061</v>
       </c>
       <c r="C15" s="55" t="n">
-        <v>0.04896</v>
+        <v>0.05218</v>
       </c>
       <c r="D15" s="55" t="n">
         <v>0.03079</v>

</xml_diff>

<commit_message>
GrowthProjection.xlsx: matrix v8 labels
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1677,7 +1677,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Matrix v7 (conditional-duration S, D-cell gold + washout-conditional rebound slice, R momentum tilt, regime-gated short book: oil in Deflation + energy equities in Stagflation behind a global include-shorts switch), monthly-only execution — intra-month mechanisms tested and rejected under honest T+1 modeling. Leveraged instruments simulated pre-2010. Out-of-sample framework validation: 1987-2007 replication. Forward: paper/ledger.csv.</t>
+          <t>Matrix v8 (AGG Reflation leverage on the energy leg — QQQ 1x + ERX 2x; conditional-duration S, D-cell gold + washout-conditional rebound slice, R momentum tilt, regime-gated short book: oil in Deflation + energy equities in Stagflation behind a global include-shorts switch), monthly-only execution — intra-month mechanisms tested and rejected under honest T+1 modeling. Leveraged instruments simulated pre-2010. Out-of-sample framework validation: 1987-2007 replication. Forward: paper/ledger.csv.</t>
         </is>
       </c>
     </row>
@@ -18302,7 +18302,7 @@
     <row r="1">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>Model Data — per-regime return statistics (matrix v7, monthly-only execution, Jun 2007–Aug 2026)</t>
+          <t>Model Data — per-regime return statistics (matrix v8, monthly-only execution, Jun 2007–Aug 2026)</t>
         </is>
       </c>
     </row>

</xml_diff>